<commit_message>
Remove student name column and invigilator line from attendance sheets
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YKBobHBYVbWbiRoSDhU7SN
</commit_message>
<xml_diff>
--- a/Lab_Attendance_Sheets_CSE_AIML.xlsx
+++ b/Lab_Attendance_Sheets_CSE_AIML.xlsx
@@ -33,51 +33,51 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'CSE_CCLab-1'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'CSE_CCLab-1'!$A$1:$E$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'CSE_CCLab-1'!$A$1:$D$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'CSE_CCLab-2'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'CSE_CCLab-2'!$A$1:$E$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'CSE_CCLab-2'!$A$1:$D$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'CSE_CISCOLab'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'CSE_CISCOLab'!$A$1:$E$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'CSE_CISCOLab'!$A$1:$D$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'CSE_CSELab-1'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'CSE_CSELab-1'!$A$1:$E$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'CSE_CSELab-1'!$A$1:$D$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'CSE_CSELab-2'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'CSE_CSELab-2'!$A$1:$E$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'CSE_CSELab-2'!$A$1:$D$31</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'CSE_CSELab-3'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'CSE_CSELab-3'!$A$1:$E$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'CSE_CSELab-3'!$A$1:$D$27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'CSE_CSELab-V'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'CSE_CSELab-V'!$A$1:$E$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'CSE_CSELab-V'!$A$1:$D$42</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'CSE_CSELab-VI'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="7">'CSE_CSELab-VI'!$A$1:$E$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">'CSE_CSELab-VI'!$A$1:$D$43</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'CSE_ITLab-1'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'CSE_ITLab-1'!$A$1:$E$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'CSE_ITLab-1'!$A$1:$D$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'CSE_ITLab-2'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'CSE_ITLab-2'!$A$1:$E$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'CSE_ITLab-2'!$A$1:$D$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'CSE_ITLab-V'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="10">'CSE_ITLab-V'!$A$1:$E$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="10">'CSE_ITLab-V'!$A$1:$D$42</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="11">'CSE_ITLab-VII'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="11">'CSE_ITLab-VII'!$A$1:$E$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'CSE_ITLab-VII'!$A$1:$D$42</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="12">'AIML_CCLab-1'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="12">'AIML_CCLab-1'!$A$1:$E$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="12">'AIML_CCLab-1'!$A$1:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="13">'AIML_CISCOLab'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="13">'AIML_CISCOLab'!$A$1:$E$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="13">'AIML_CISCOLab'!$A$1:$D$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="14">'AIML_CSELab-1'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="14">'AIML_CSELab-1'!$A$1:$E$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="14">'AIML_CSELab-1'!$A$1:$D$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="15">'AIML_CSELab-2'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="15">'AIML_CSELab-2'!$A$1:$E$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="15">'AIML_CSELab-2'!$A$1:$D$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="16">'AIML_CSELab-3'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="16">'AIML_CSELab-3'!$A$1:$E$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="16">'AIML_CSELab-3'!$A$1:$D$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="17">'AIML_CSELab-V'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="17">'AIML_CSELab-V'!$A$1:$E$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="17">'AIML_CSELab-V'!$A$1:$D$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="18">'AIML_CSELab-VI'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="18">'AIML_CSELab-VI'!$A$1:$E$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="18">'AIML_CSELab-VI'!$A$1:$D$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="19">'AIML_ITLab-1'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="19">'AIML_ITLab-1'!$A$1:$E$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="19">'AIML_ITLab-1'!$A$1:$D$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="20">'AIML_ITLab-2'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="20">'AIML_ITLab-2'!$A$1:$E$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="20">'AIML_ITLab-2'!$A$1:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="21">'AIML_ITLab-V'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="21">'AIML_ITLab-V'!$A$1:$E$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="21">'AIML_ITLab-V'!$A$1:$D$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="22">'AIML_ITLab-VII'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="22">'AIML_ITLab-VII'!$A$1:$E$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="22">'AIML_ITLab-VII'!$A$1:$D$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -533,14 +533,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -598,15 +597,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -623,7 +617,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -636,7 +629,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -649,7 +641,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -662,7 +653,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -675,7 +665,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -688,7 +677,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -697,21 +685,14 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -724,14 +705,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -789,15 +769,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -814,7 +789,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -827,7 +801,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -840,7 +813,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -853,7 +825,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -866,7 +837,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -879,7 +849,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -888,21 +857,14 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -915,14 +877,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -980,15 +941,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -1005,7 +961,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -1018,7 +973,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -1031,7 +985,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -1044,7 +997,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -1057,7 +1009,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -1070,7 +1021,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -1083,7 +1033,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -1096,7 +1045,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -1109,7 +1057,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -1122,7 +1069,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -1135,7 +1081,6 @@
       </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -1148,7 +1093,6 @@
       </c>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -1161,7 +1105,6 @@
       </c>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="6" t="n">
@@ -1174,7 +1117,6 @@
       </c>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -1187,7 +1129,6 @@
       </c>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="6" t="n">
@@ -1200,7 +1141,6 @@
       </c>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="6" t="n">
@@ -1213,7 +1153,6 @@
       </c>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="6" t="n">
@@ -1226,7 +1165,6 @@
       </c>
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="6" t="n">
@@ -1239,7 +1177,6 @@
       </c>
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="6" t="n">
@@ -1252,7 +1189,6 @@
       </c>
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="6" t="n">
@@ -1265,7 +1201,6 @@
       </c>
       <c r="C29" s="7" t="n"/>
       <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="6" t="n">
@@ -1278,7 +1213,6 @@
       </c>
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="6" t="n">
@@ -1291,7 +1225,6 @@
       </c>
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="6" t="n">
@@ -1304,7 +1237,6 @@
       </c>
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="6" t="n">
@@ -1317,7 +1249,6 @@
       </c>
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="6" t="n">
@@ -1330,7 +1261,6 @@
       </c>
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="6" t="n">
@@ -1343,7 +1273,6 @@
       </c>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="6" t="n">
@@ -1356,7 +1285,6 @@
       </c>
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="6" t="n">
@@ -1369,7 +1297,6 @@
       </c>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
-      <c r="E37" s="7" t="n"/>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="6" t="n">
@@ -1382,7 +1309,6 @@
       </c>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
     </row>
     <row r="39" ht="24" customHeight="1">
       <c r="A39" s="6" t="n">
@@ -1395,7 +1321,6 @@
       </c>
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1404,21 +1329,14 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -1431,14 +1349,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1496,15 +1413,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -1521,7 +1433,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -1534,7 +1445,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -1547,7 +1457,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -1560,7 +1469,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -1573,7 +1481,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -1586,7 +1493,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -1599,7 +1505,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -1612,7 +1517,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -1625,7 +1529,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -1638,7 +1541,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -1651,7 +1553,6 @@
       </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -1664,7 +1565,6 @@
       </c>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -1677,7 +1577,6 @@
       </c>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="6" t="n">
@@ -1690,7 +1589,6 @@
       </c>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -1703,7 +1601,6 @@
       </c>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="6" t="n">
@@ -1716,7 +1613,6 @@
       </c>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="6" t="n">
@@ -1729,7 +1625,6 @@
       </c>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="6" t="n">
@@ -1742,7 +1637,6 @@
       </c>
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="6" t="n">
@@ -1755,7 +1649,6 @@
       </c>
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="6" t="n">
@@ -1768,7 +1661,6 @@
       </c>
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="6" t="n">
@@ -1781,7 +1673,6 @@
       </c>
       <c r="C29" s="7" t="n"/>
       <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="6" t="n">
@@ -1794,7 +1685,6 @@
       </c>
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="6" t="n">
@@ -1807,7 +1697,6 @@
       </c>
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="6" t="n">
@@ -1820,7 +1709,6 @@
       </c>
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="6" t="n">
@@ -1833,7 +1721,6 @@
       </c>
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="6" t="n">
@@ -1846,7 +1733,6 @@
       </c>
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="6" t="n">
@@ -1859,7 +1745,6 @@
       </c>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="6" t="n">
@@ -1872,7 +1757,6 @@
       </c>
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="6" t="n">
@@ -1885,7 +1769,6 @@
       </c>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
-      <c r="E37" s="7" t="n"/>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="6" t="n">
@@ -1898,7 +1781,6 @@
       </c>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
     </row>
     <row r="39" ht="24" customHeight="1">
       <c r="A39" s="6" t="n">
@@ -1911,7 +1793,6 @@
       </c>
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1920,21 +1801,14 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -1947,14 +1821,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2012,15 +1885,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2037,7 +1905,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -2050,7 +1917,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -2063,7 +1929,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2072,21 +1937,14 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2099,14 +1957,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2164,15 +2021,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2189,7 +2041,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -2202,7 +2053,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -2215,7 +2065,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -2228,7 +2077,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -2241,7 +2089,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2250,21 +2097,14 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2277,14 +2117,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2342,15 +2181,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2367,7 +2201,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -2380,7 +2213,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -2393,7 +2225,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -2406,7 +2237,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -2419,7 +2249,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2428,21 +2257,14 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2455,14 +2277,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2520,15 +2341,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2545,7 +2361,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -2558,7 +2373,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -2571,7 +2385,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -2584,7 +2397,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -2597,7 +2409,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2606,21 +2417,14 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2633,14 +2437,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2698,15 +2501,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2723,7 +2521,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -2736,7 +2533,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -2749,7 +2545,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -2762,7 +2557,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -2775,7 +2569,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2784,21 +2577,14 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2811,14 +2597,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2876,15 +2661,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2901,7 +2681,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -2914,7 +2693,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -2927,7 +2705,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -2940,7 +2717,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -2953,7 +2729,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -2966,7 +2741,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -2979,7 +2753,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -2992,7 +2765,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -3005,7 +2777,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -3018,7 +2789,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -3031,7 +2801,6 @@
       </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3040,21 +2809,14 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -3067,14 +2829,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3132,15 +2893,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -3157,7 +2913,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -3170,7 +2925,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -3183,7 +2937,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -3196,7 +2949,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -3209,7 +2961,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -3222,7 +2973,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -3235,7 +2985,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -3248,7 +2997,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -3261,7 +3009,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -3274,7 +3021,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3283,21 +3029,14 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -3310,14 +3049,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3375,15 +3113,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -3400,7 +3133,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -3413,7 +3145,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -3426,7 +3157,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -3439,7 +3169,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -3452,7 +3181,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -3465,7 +3193,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -3478,7 +3205,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3487,21 +3213,14 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -3514,14 +3233,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3579,15 +3297,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -3604,7 +3317,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -3617,7 +3329,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -3630,7 +3341,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -3643,7 +3353,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3652,21 +3361,14 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -3679,14 +3381,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3744,15 +3445,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -3769,7 +3465,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -3782,7 +3477,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -3795,7 +3489,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3804,21 +3497,14 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -3831,14 +3517,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3896,15 +3581,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -3921,7 +3601,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -3934,7 +3613,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -3947,7 +3625,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -3960,7 +3637,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -3973,7 +3649,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -3986,7 +3661,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -3999,7 +3673,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -4012,7 +3685,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -4025,7 +3697,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -4038,7 +3709,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -4051,7 +3721,6 @@
       </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4060,21 +3729,14 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -4087,14 +3749,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4152,15 +3813,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -4177,7 +3833,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -4190,7 +3845,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -4203,7 +3857,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -4216,7 +3869,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -4229,7 +3881,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -4242,7 +3893,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -4255,7 +3905,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -4268,7 +3917,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -4281,7 +3929,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -4294,7 +3941,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4303,21 +3949,14 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -4330,14 +3969,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4395,15 +4033,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -4420,7 +4053,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -4433,7 +4065,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -4446,7 +4077,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -4459,7 +4089,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -4472,7 +4101,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -4485,7 +4113,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -4498,7 +4125,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -4511,7 +4137,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -4524,7 +4149,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -4537,7 +4161,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4546,21 +4169,14 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -4573,14 +4189,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4638,15 +4253,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -4663,7 +4273,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -4676,7 +4285,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -4689,7 +4297,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -4702,7 +4309,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -4715,7 +4321,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -4728,7 +4333,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -4741,7 +4345,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -4754,7 +4357,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -4767,7 +4369,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -4780,7 +4381,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -4793,7 +4393,6 @@
       </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -4806,7 +4405,6 @@
       </c>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -4819,7 +4417,6 @@
       </c>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4828,21 +4425,14 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -4855,14 +4445,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4920,15 +4509,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -4945,7 +4529,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -4958,7 +4541,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -4971,7 +4553,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -4984,7 +4565,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -4997,7 +4577,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -5010,7 +4589,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -5023,7 +4601,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -5036,7 +4613,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -5049,7 +4625,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -5062,7 +4637,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -5075,7 +4649,6 @@
       </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -5088,7 +4661,6 @@
       </c>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -5101,7 +4673,6 @@
       </c>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="6" t="n">
@@ -5114,7 +4685,6 @@
       </c>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -5127,7 +4697,6 @@
       </c>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="6" t="n">
@@ -5140,7 +4709,6 @@
       </c>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="6" t="n">
@@ -5153,7 +4721,6 @@
       </c>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="6" t="n">
@@ -5166,7 +4733,6 @@
       </c>
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="6" t="n">
@@ -5179,7 +4745,6 @@
       </c>
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="6" t="n">
@@ -5192,7 +4757,6 @@
       </c>
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5201,21 +4765,14 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -5228,14 +4785,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5293,15 +4849,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -5318,7 +4869,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -5331,7 +4881,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -5344,7 +4893,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -5357,7 +4905,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -5370,7 +4917,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -5383,7 +4929,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -5396,7 +4941,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -5409,7 +4953,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -5422,7 +4965,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -5435,7 +4977,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -5448,7 +4989,6 @@
       </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -5461,7 +5001,6 @@
       </c>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -5474,7 +5013,6 @@
       </c>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="6" t="n">
@@ -5487,7 +5025,6 @@
       </c>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -5500,7 +5037,6 @@
       </c>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="6" t="n">
@@ -5513,7 +5049,6 @@
       </c>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5522,21 +5057,14 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -5549,14 +5077,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5614,15 +5141,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -5639,7 +5161,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -5652,7 +5173,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -5665,7 +5185,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -5678,7 +5197,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -5691,7 +5209,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -5704,7 +5221,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -5717,7 +5233,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -5730,7 +5245,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -5743,7 +5257,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -5756,7 +5269,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -5769,7 +5281,6 @@
       </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -5782,7 +5293,6 @@
       </c>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -5795,7 +5305,6 @@
       </c>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="6" t="n">
@@ -5808,7 +5317,6 @@
       </c>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -5821,7 +5329,6 @@
       </c>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="6" t="n">
@@ -5834,7 +5341,6 @@
       </c>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="6" t="n">
@@ -5847,7 +5353,6 @@
       </c>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="6" t="n">
@@ -5860,7 +5365,6 @@
       </c>
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="6" t="n">
@@ -5873,7 +5377,6 @@
       </c>
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="6" t="n">
@@ -5886,7 +5389,6 @@
       </c>
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="6" t="n">
@@ -5899,7 +5401,6 @@
       </c>
       <c r="C29" s="7" t="n"/>
       <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="6" t="n">
@@ -5912,7 +5413,6 @@
       </c>
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="6" t="n">
@@ -5925,7 +5425,6 @@
       </c>
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="6" t="n">
@@ -5938,7 +5437,6 @@
       </c>
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="6" t="n">
@@ -5951,7 +5449,6 @@
       </c>
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="6" t="n">
@@ -5964,7 +5461,6 @@
       </c>
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="6" t="n">
@@ -5977,7 +5473,6 @@
       </c>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="6" t="n">
@@ -5990,7 +5485,6 @@
       </c>
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="6" t="n">
@@ -6003,7 +5497,6 @@
       </c>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
-      <c r="E37" s="7" t="n"/>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="6" t="n">
@@ -6016,7 +5509,6 @@
       </c>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
     </row>
     <row r="39" ht="24" customHeight="1">
       <c r="A39" s="6" t="n">
@@ -6029,7 +5521,6 @@
       </c>
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6038,21 +5529,14 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -6065,14 +5549,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6130,15 +5613,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -6155,7 +5633,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -6168,7 +5645,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -6181,7 +5657,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -6194,7 +5669,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -6207,7 +5681,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -6220,7 +5693,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -6233,7 +5705,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -6246,7 +5717,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -6259,7 +5729,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -6272,7 +5741,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -6285,7 +5753,6 @@
       </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -6298,7 +5765,6 @@
       </c>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -6311,7 +5777,6 @@
       </c>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="6" t="n">
@@ -6324,7 +5789,6 @@
       </c>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -6337,7 +5801,6 @@
       </c>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="6" t="n">
@@ -6350,7 +5813,6 @@
       </c>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="6" t="n">
@@ -6363,7 +5825,6 @@
       </c>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="6" t="n">
@@ -6376,7 +5837,6 @@
       </c>
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="6" t="n">
@@ -6389,7 +5849,6 @@
       </c>
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="6" t="n">
@@ -6402,7 +5861,6 @@
       </c>
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="6" t="n">
@@ -6415,7 +5873,6 @@
       </c>
       <c r="C29" s="7" t="n"/>
       <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="6" t="n">
@@ -6428,7 +5885,6 @@
       </c>
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="6" t="n">
@@ -6441,7 +5897,6 @@
       </c>
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="6" t="n">
@@ -6454,7 +5909,6 @@
       </c>
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="6" t="n">
@@ -6467,7 +5921,6 @@
       </c>
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="6" t="n">
@@ -6480,7 +5933,6 @@
       </c>
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="6" t="n">
@@ -6493,7 +5945,6 @@
       </c>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="6" t="n">
@@ -6506,7 +5957,6 @@
       </c>
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="6" t="n">
@@ -6519,7 +5969,6 @@
       </c>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
-      <c r="E37" s="7" t="n"/>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="6" t="n">
@@ -6532,7 +5981,6 @@
       </c>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
     </row>
     <row r="39" ht="24" customHeight="1">
       <c r="A39" s="6" t="n">
@@ -6545,7 +5993,6 @@
       </c>
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
     </row>
     <row r="40" ht="24" customHeight="1">
       <c r="A40" s="6" t="n">
@@ -6558,7 +6005,6 @@
       </c>
       <c r="C40" s="7" t="n"/>
       <c r="D40" s="7" t="n"/>
-      <c r="E40" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6567,21 +6013,14 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -6594,14 +6033,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6659,15 +6097,10 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student Name</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -6684,7 +6117,6 @@
       </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -6697,7 +6129,6 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -6710,7 +6141,6 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -6723,7 +6153,6 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -6736,7 +6165,6 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -6749,7 +6177,6 @@
       </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -6762,7 +6189,6 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -6775,7 +6201,6 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -6788,7 +6213,6 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -6801,7 +6225,6 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6810,21 +6233,14 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Invigilator Name &amp; Signature: ______________________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>